<commit_message>
Signed-off-by: sonali kulkarni <sonalikulkarni3697@gmail.com>
</commit_message>
<xml_diff>
--- a/Assesment/Assesment.xlsx
+++ b/Assesment/Assesment.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="273">
   <si>
     <t>Test case ID</t>
   </si>
@@ -153,13 +153,715 @@
     <t>username-
 password-
 clicl login</t>
+  </si>
+  <si>
+    <t>Check Website URL</t>
+  </si>
+  <si>
+    <t>Internet, working website, browser</t>
+  </si>
+  <si>
+    <t>1. Enter URL 2. Press Enter</t>
+  </si>
+  <si>
+    <t>Application should open successfully</t>
+  </si>
+  <si>
+    <t>Application opens as expected</t>
+  </si>
+  <si>
+    <t>Check Search Multiplex Field Visibility</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Search Multiplex by Name</t>
+  </si>
+  <si>
+    <t>Browse Multiplex List</t>
+  </si>
+  <si>
+    <t>Multiplex detail page should open</t>
+  </si>
+  <si>
+    <t>Seat layout page should open</t>
+  </si>
+  <si>
+    <t>Proceed to Payment Button</t>
+  </si>
+  <si>
+    <t>1. Click Proceed to Payment</t>
+  </si>
+  <si>
+    <t>Payment page should open</t>
+  </si>
+  <si>
+    <t>Payment completed</t>
+  </si>
+  <si>
+    <t>Booking confirmation page should display</t>
+  </si>
+  <si>
+    <t>1. Locate search bar</t>
+  </si>
+  <si>
+    <t>Search field should be visible</t>
+  </si>
+  <si>
+    <t>Search field visible</t>
+  </si>
+  <si>
+    <t>1. Enter multiplex name 2. Click search</t>
+  </si>
+  <si>
+    <t>“PVR Icon”</t>
+  </si>
+  <si>
+    <t>Search results should display</t>
+  </si>
+  <si>
+    <t>Results displayed</t>
+  </si>
+  <si>
+    <t>Search Multiplex with Partial Name</t>
+  </si>
+  <si>
+    <t>1. Enter partial name 2. Click search</t>
+  </si>
+  <si>
+    <t>“INO”</t>
+  </si>
+  <si>
+    <t>Suggested multiplex list should appear</t>
+  </si>
+  <si>
+    <t>Suggestions appear</t>
+  </si>
+  <si>
+    <t>Search Multiplex with Invalid Name</t>
+  </si>
+  <si>
+    <t>1. Enter invalid name 2. Click search</t>
+  </si>
+  <si>
+    <t>“XYZ123”</t>
+  </si>
+  <si>
+    <t>No results message should display</t>
+  </si>
+  <si>
+    <t>No results shown</t>
+  </si>
+  <si>
+    <t>1. Click Browse Multiplex</t>
+  </si>
+  <si>
+    <t>Multiplex list should display</t>
+  </si>
+  <si>
+    <t>List displayed</t>
+  </si>
+  <si>
+    <t>Scroll Multiplex List</t>
+  </si>
+  <si>
+    <t>1. Scroll list</t>
+  </si>
+  <si>
+    <t>More multiplexes should load</t>
+  </si>
+  <si>
+    <t>Data loads</t>
+  </si>
+  <si>
+    <t>Select Multiplex from List</t>
+  </si>
+  <si>
+    <t>1. Click multiplex name</t>
+  </si>
+  <si>
+    <t>“INOX Mall Road”</t>
+  </si>
+  <si>
+    <t>Page opens</t>
+  </si>
+  <si>
+    <t>View Movie List in Multiplex</t>
+  </si>
+  <si>
+    <t>1. Check movie listing</t>
+  </si>
+  <si>
+    <t>Movie list should display</t>
+  </si>
+  <si>
+    <t>Movies displayed</t>
+  </si>
+  <si>
+    <t>Select Movie</t>
+  </si>
+  <si>
+    <t>1. Click movie name</t>
+  </si>
+  <si>
+    <t>“Movie A”</t>
+  </si>
+  <si>
+    <t>Show timings should display</t>
+  </si>
+  <si>
+    <t>Timings visible</t>
+  </si>
+  <si>
+    <t>Select Show Timing</t>
+  </si>
+  <si>
+    <t>1. Select show time</t>
+  </si>
+  <si>
+    <t>Layout opens</t>
+  </si>
+  <si>
+    <t>Verify Seat Layout Load</t>
+  </si>
+  <si>
+    <t>1. Wait for layout load</t>
+  </si>
+  <si>
+    <t>Seat layout should load</t>
+  </si>
+  <si>
+    <t>Layout displayed</t>
+  </si>
+  <si>
+    <t>Select Single Seat</t>
+  </si>
+  <si>
+    <t>1. Click available seat</t>
+  </si>
+  <si>
+    <t>A-5</t>
+  </si>
+  <si>
+    <t>Seat should get selected</t>
+  </si>
+  <si>
+    <t>Seat highlighted</t>
+  </si>
+  <si>
+    <t>Select Multiple Seats</t>
+  </si>
+  <si>
+    <t>1. Select 2 seats</t>
+  </si>
+  <si>
+    <t>A-5, A-6</t>
+  </si>
+  <si>
+    <t>Multiple seats should be selected</t>
+  </si>
+  <si>
+    <t>Seats selected</t>
+  </si>
+  <si>
+    <t>Select Already Booked Seat</t>
+  </si>
+  <si>
+    <t>1. Click booked seat</t>
+  </si>
+  <si>
+    <t>Seat B-7</t>
+  </si>
+  <si>
+    <t>System should not allow selection</t>
+  </si>
+  <si>
+    <t>Selection restricted</t>
+  </si>
+  <si>
+    <t>Deselect Selected Seat</t>
+  </si>
+  <si>
+    <t>1. Click same seat again</t>
+  </si>
+  <si>
+    <t>Seat should get deselected</t>
+  </si>
+  <si>
+    <t>Seat deselected</t>
+  </si>
+  <si>
+    <t>Check Ticket Price Update</t>
+  </si>
+  <si>
+    <t>1. Select seat 2. Observe price</t>
+  </si>
+  <si>
+    <t>Price should update dynamically</t>
+  </si>
+  <si>
+    <t>Price updated</t>
+  </si>
+  <si>
+    <t>1. Click Proceed to Pay</t>
+  </si>
+  <si>
+    <t>Payment page opens</t>
+  </si>
+  <si>
+    <t>Proceed Without Seat Selection</t>
+  </si>
+  <si>
+    <t>System should show validation message</t>
+  </si>
+  <si>
+    <t>Error message displayed</t>
+  </si>
+  <si>
+    <t>Apply Coupon Code</t>
+  </si>
+  <si>
+    <t>Payment page open</t>
+  </si>
+  <si>
+    <t>1. Enter coupon 2. Apply</t>
+  </si>
+  <si>
+    <t>SAVE50</t>
+  </si>
+  <si>
+    <t>Discount should be applied</t>
+  </si>
+  <si>
+    <t>Discount applied</t>
+  </si>
+  <si>
+    <t>Invalid Coupon Code</t>
+  </si>
+  <si>
+    <t>1. Enter invalid code</t>
+  </si>
+  <si>
+    <t>INVALID10</t>
+  </si>
+  <si>
+    <t>Error message should display</t>
+  </si>
+  <si>
+    <t>Error displayed</t>
+  </si>
+  <si>
+    <t>Select Payment Method</t>
+  </si>
+  <si>
+    <t>1. Choose UPI/Card</t>
+  </si>
+  <si>
+    <t>UPI</t>
+  </si>
+  <si>
+    <t>Selected mode should activate</t>
+  </si>
+  <si>
+    <t>Mode activated</t>
+  </si>
+  <si>
+    <t>Complete Successful Payment</t>
+  </si>
+  <si>
+    <t>1. Enter payment info 2. Pay</t>
+  </si>
+  <si>
+    <t>UPI/Card</t>
+  </si>
+  <si>
+    <t>Ticket confirmed</t>
+  </si>
+  <si>
+    <t>Booking Confirmation Email/SMS</t>
+  </si>
+  <si>
+    <t>Payment successful</t>
+  </si>
+  <si>
+    <t>1. Check email/SMS</t>
+  </si>
+  <si>
+    <t>Registered email/number</t>
+  </si>
+  <si>
+    <t>Confirmation message should be received</t>
+  </si>
+  <si>
+    <t>Confirmation received</t>
+  </si>
+  <si>
+    <t>Logout and Re-Login Ticket Visible</t>
+  </si>
+  <si>
+    <t>1. Logout 2. Login again 3. Check bookings</t>
+  </si>
+  <si>
+    <t>User credentials</t>
+  </si>
+  <si>
+    <t>Ticket should appear in bookings history</t>
+  </si>
+  <si>
+    <t>Ticket visible</t>
+  </si>
+  <si>
+    <t>Verify Payment Page Navigation</t>
+  </si>
+  <si>
+    <t>Seat selected, user logged in</t>
+  </si>
+  <si>
+    <t>User should navigate to payment page</t>
+  </si>
+  <si>
+    <t>Validate Payment Methods Display</t>
+  </si>
+  <si>
+    <t>On payment page</t>
+  </si>
+  <si>
+    <t>1. Check payment method list</t>
+  </si>
+  <si>
+    <t>All payment methods should display</t>
+  </si>
+  <si>
+    <t>Methods visible</t>
+  </si>
+  <si>
+    <t>Select UPI Payment Method</t>
+  </si>
+  <si>
+    <t>1. Select UPI option</t>
+  </si>
+  <si>
+    <t>UPI fields should activate</t>
+  </si>
+  <si>
+    <t>UPI enabled</t>
+  </si>
+  <si>
+    <t>Select Debit/Credit Card Option</t>
+  </si>
+  <si>
+    <t>1. Select Card option</t>
+  </si>
+  <si>
+    <t>Card</t>
+  </si>
+  <si>
+    <t>Card fields should activate</t>
+  </si>
+  <si>
+    <t>Card form enabled</t>
+  </si>
+  <si>
+    <t>Enter Valid Card Details</t>
+  </si>
+  <si>
+    <t>Card option selected</t>
+  </si>
+  <si>
+    <t>1. Enter card details 2. Click Pay</t>
+  </si>
+  <si>
+    <t>Valid card details</t>
+  </si>
+  <si>
+    <t>Payment should be processed</t>
+  </si>
+  <si>
+    <t>Payment success</t>
+  </si>
+  <si>
+    <t>Enter Invalid Card Number</t>
+  </si>
+  <si>
+    <t>1. Enter wrong card number 2. Click Pay</t>
+  </si>
+  <si>
+    <t>1111 2222 3333</t>
+  </si>
+  <si>
+    <t>Error message should appear</t>
+  </si>
+  <si>
+    <t>Expired Card Validation</t>
+  </si>
+  <si>
+    <t>1. Enter expired card date</t>
+  </si>
+  <si>
+    <t>Expiry 01/2023</t>
+  </si>
+  <si>
+    <t>System should restrict transaction</t>
+  </si>
+  <si>
+    <t>Validation message shown</t>
+  </si>
+  <si>
+    <t>Incorrect CVV Handling</t>
+  </si>
+  <si>
+    <t>1. Enter wrong CVV</t>
+  </si>
+  <si>
+    <t>CVV error displayed</t>
+  </si>
+  <si>
+    <t>Payment Timeout Scenario</t>
+  </si>
+  <si>
+    <t>Payment initiated</t>
+  </si>
+  <si>
+    <t>1. Wait for session timeout</t>
+  </si>
+  <si>
+    <t>Transaction should fail gracefully</t>
+  </si>
+  <si>
+    <t>Timeout handled</t>
+  </si>
+  <si>
+    <t>Retry Payment After Failure</t>
+  </si>
+  <si>
+    <t>Payment failed</t>
+  </si>
+  <si>
+    <t>1. Click Retry Payment</t>
+  </si>
+  <si>
+    <t>User should be able to retry</t>
+  </si>
+  <si>
+    <t>Retry works</t>
+  </si>
+  <si>
+    <t>UPI Payment Success</t>
+  </si>
+  <si>
+    <t>UPI selected</t>
+  </si>
+  <si>
+    <t>1. Enter UPI ID 2. Approve payment</t>
+  </si>
+  <si>
+    <t>test@upi</t>
+  </si>
+  <si>
+    <t>Payment should succeed</t>
+  </si>
+  <si>
+    <t>Success message displayed</t>
+  </si>
+  <si>
+    <t>Invalid UPI ID</t>
+  </si>
+  <si>
+    <t>1. Enter invalid UPI</t>
+  </si>
+  <si>
+    <t>abc@xyz</t>
+  </si>
+  <si>
+    <t>Invalid UPI error</t>
+  </si>
+  <si>
+    <t>Net Banking Payment Success</t>
+  </si>
+  <si>
+    <t>Net banking selected</t>
+  </si>
+  <si>
+    <t>1. Select bank 2. Login 3. Pay</t>
+  </si>
+  <si>
+    <t>SBI Net Banking</t>
+  </si>
+  <si>
+    <t>Payment should complete</t>
+  </si>
+  <si>
+    <t>Success confirmation</t>
+  </si>
+  <si>
+    <t>Cancel Payment from Bank Page</t>
+  </si>
+  <si>
+    <t>On bank page</t>
+  </si>
+  <si>
+    <t>1. Click Cancel</t>
+  </si>
+  <si>
+    <t>Booking should not be confirmed</t>
+  </si>
+  <si>
+    <t>Payment cancelled</t>
+  </si>
+  <si>
+    <t>Check Payment Amount Display</t>
+  </si>
+  <si>
+    <t>1. Verify final amount</t>
+  </si>
+  <si>
+    <t>Amount with tax</t>
+  </si>
+  <si>
+    <t>Correct price should display</t>
+  </si>
+  <si>
+    <t>Price correct</t>
+  </si>
+  <si>
+    <t>Apply Valid Coupon Code</t>
+  </si>
+  <si>
+    <t>Discount should apply</t>
+  </si>
+  <si>
+    <t>Discount visible</t>
+  </si>
+  <si>
+    <t>Apply Invalid Coupon Code</t>
+  </si>
+  <si>
+    <t>1. Enter invalid coupon</t>
+  </si>
+  <si>
+    <t>XYZ10</t>
+  </si>
+  <si>
+    <t>Validation message should display</t>
+  </si>
+  <si>
+    <t>Invalid coupon alert</t>
+  </si>
+  <si>
+    <t>Remove Applied Coupon</t>
+  </si>
+  <si>
+    <t>Coupon applied</t>
+  </si>
+  <si>
+    <t>1. Click Remove Coupon</t>
+  </si>
+  <si>
+    <t>Total amount should revert</t>
+  </si>
+  <si>
+    <t>Amount reverted</t>
+  </si>
+  <si>
+    <t>GST/Taxes Calculation</t>
+  </si>
+  <si>
+    <t>Amount displayed</t>
+  </si>
+  <si>
+    <t>1. Verify tax calculation</t>
+  </si>
+  <si>
+    <t>Ticket + GST</t>
+  </si>
+  <si>
+    <t>Correct tax should calculate</t>
+  </si>
+  <si>
+    <t>Tax accurate</t>
+  </si>
+  <si>
+    <t>Download Payment Invoice</t>
+  </si>
+  <si>
+    <t>1. Click Download Invoice</t>
+  </si>
+  <si>
+    <t>Invoice should download</t>
+  </si>
+  <si>
+    <t>Invoice downloaded</t>
+  </si>
+  <si>
+    <t>Payment Confirmation Page</t>
+  </si>
+  <si>
+    <t>1. Observe confirmation page</t>
+  </si>
+  <si>
+    <t>Confirmation page should display</t>
+  </si>
+  <si>
+    <t>Duplicate Payment Prevention</t>
+  </si>
+  <si>
+    <t>Payment already completed</t>
+  </si>
+  <si>
+    <t>1. Click Pay again</t>
+  </si>
+  <si>
+    <t>System should block duplicate charge</t>
+  </si>
+  <si>
+    <t>Duplicate prevented</t>
+  </si>
+  <si>
+    <t>Wallet Payment Option</t>
+  </si>
+  <si>
+    <t>Wallet enabled</t>
+  </si>
+  <si>
+    <t>1. Select Wallet 2. Pay</t>
+  </si>
+  <si>
+    <t>Paytm Wallet</t>
+  </si>
+  <si>
+    <t>Low Wallet Balance Handling</t>
+  </si>
+  <si>
+    <t>Wallet payment selected</t>
+  </si>
+  <si>
+    <t>1. Try paying with low balance</t>
+  </si>
+  <si>
+    <t>₹10</t>
+  </si>
+  <si>
+    <t>Insufficient balance alert</t>
+  </si>
+  <si>
+    <t>Auto-Redirect to Confirmation</t>
+  </si>
+  <si>
+    <t>1. Wait after payment completion</t>
+  </si>
+  <si>
+    <t>System should auto-redirect to booking summary</t>
+  </si>
+  <si>
+    <t>Redirect successful</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,6 +881,13 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -205,7 +914,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -216,6 +925,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -229,6 +945,101 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/activeX/activeX1.xml><?xml version="1.0" encoding="utf-8"?>
+<ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{5512D124-5CC6-11CF-8D67-00AA00BDCE1D}" ax:persistence="persistStream" r:id="rId1"/>
+</file>
+
+<file path=xl/activeX/activeX2.xml><?xml version="1.0" encoding="utf-8"?>
+<ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{5512D124-5CC6-11CF-8D67-00AA00BDCE1D}" ax:persistence="persistStream" r:id="rId1"/>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>52</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>4</xdr:col>
+          <xdr:colOff>514350</xdr:colOff>
+          <xdr:row>53</xdr:row>
+          <xdr:rowOff>352425</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1025" name="Control 1" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1025"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>0</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>52</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>523875</xdr:colOff>
+          <xdr:row>53</xdr:row>
+          <xdr:rowOff>352425</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1026" name="Control 2" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1026"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -517,8 +1328,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
@@ -531,85 +1343,85 @@
     <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="105" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>10</v>
+      <c r="C2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>41</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="G2" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="105" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>16</v>
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>18</v>
+        <v>10</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>14</v>
@@ -618,44 +1430,44 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>14</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>9</v>
@@ -664,7 +1476,7 @@
         <v>22</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>23</v>
@@ -673,18 +1485,18 @@
         <v>14</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>9</v>
@@ -693,7 +1505,7 @@
         <v>22</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>23</v>
@@ -705,15 +1517,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>9</v>
@@ -721,8 +1533,8 @@
       <c r="E7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>29</v>
+      <c r="F7" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>23</v>
@@ -734,15 +1546,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>9</v>
@@ -751,7 +1563,7 @@
         <v>22</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>23</v>
@@ -763,15 +1575,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>9</v>
@@ -780,7 +1592,7 @@
         <v>22</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>23</v>
@@ -792,15 +1604,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="105" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>9</v>
@@ -808,8 +1620,8 @@
       <c r="E10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>36</v>
+      <c r="F10" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>23</v>
@@ -821,15 +1633,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>9</v>
@@ -838,7 +1650,7 @@
         <v>22</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>23</v>
@@ -850,23 +1662,1591 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="105" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12">
         <v>11</v>
       </c>
+      <c r="C12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J13" s="4"/>
+    </row>
+    <row r="14" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>13</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+    </row>
+    <row r="15" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>14</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+    </row>
+    <row r="16" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+    </row>
+    <row r="17" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>16</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+    </row>
+    <row r="18" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>17</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+    </row>
+    <row r="19" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="4">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>18</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+    </row>
+    <row r="20" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>19</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+    </row>
+    <row r="21" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="4">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>20</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+    </row>
+    <row r="22" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>21</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F22" s="5">
+        <v>0.8125</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+    </row>
+    <row r="23" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="4">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>22</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+    </row>
+    <row r="24" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>23</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+    </row>
+    <row r="25" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>24</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+    </row>
+    <row r="26" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>25</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+    </row>
+    <row r="27" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="4">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>26</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+    </row>
+    <row r="28" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>27</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+    </row>
+    <row r="29" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A29" s="4">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>28</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+    </row>
+    <row r="30" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>29</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
+    </row>
+    <row r="31" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="4">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>30</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="I31" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J31" s="4"/>
+      <c r="K31" s="4"/>
+    </row>
+    <row r="32" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>31</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4"/>
+    </row>
+    <row r="33" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A33" s="4">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>32</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
+    </row>
+    <row r="34" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>33</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
+    </row>
+    <row r="35" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A35" s="4">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>34</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J35" s="4"/>
+      <c r="K35" s="4"/>
+    </row>
+    <row r="36" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>35</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
+    </row>
+    <row r="37" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A37" s="4">
+        <v>36</v>
+      </c>
+      <c r="B37" s="4">
+        <v>36</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="I37" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+      <c r="A38" s="4">
+        <v>37</v>
+      </c>
+      <c r="B38" s="4">
+        <v>37</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J38" s="4"/>
+    </row>
+    <row r="39" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A39" s="4">
+        <v>38</v>
+      </c>
+      <c r="B39" s="4">
+        <v>38</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J39" s="4"/>
+    </row>
+    <row r="40" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A40" s="4">
+        <v>39</v>
+      </c>
+      <c r="B40" s="4">
+        <v>39</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J40" s="4"/>
+    </row>
+    <row r="41" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A41" s="4">
+        <v>40</v>
+      </c>
+      <c r="B41" s="4">
+        <v>40</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J41" s="4"/>
+    </row>
+    <row r="42" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A42" s="4">
+        <v>41</v>
+      </c>
+      <c r="B42" s="4">
+        <v>41</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J42" s="4"/>
+    </row>
+    <row r="43" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A43" s="4">
+        <v>42</v>
+      </c>
+      <c r="B43" s="4">
+        <v>42</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="I43" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J43" s="4"/>
+    </row>
+    <row r="44" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A44" s="4">
+        <v>43</v>
+      </c>
+      <c r="B44" s="4">
+        <v>43</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="F44" s="4">
+        <v>0</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="H44" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="I44" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J44" s="4"/>
+    </row>
+    <row r="45" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A45" s="4">
+        <v>44</v>
+      </c>
+      <c r="B45" s="4">
+        <v>44</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J45" s="4"/>
+    </row>
+    <row r="46" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A46" s="4">
+        <v>45</v>
+      </c>
+      <c r="B46" s="4">
+        <v>45</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="I46" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J46" s="4"/>
+    </row>
+    <row r="47" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A47" s="4">
+        <v>46</v>
+      </c>
+      <c r="B47" s="4">
+        <v>46</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J47" s="4"/>
+    </row>
+    <row r="48" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A48" s="4">
+        <v>47</v>
+      </c>
+      <c r="B48" s="4">
+        <v>47</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="I48" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J48" s="4"/>
+    </row>
+    <row r="49" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A49" s="4">
+        <v>48</v>
+      </c>
+      <c r="B49" s="4">
+        <v>48</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="I49" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J49" s="4"/>
+    </row>
+    <row r="50" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A50" s="4">
+        <v>49</v>
+      </c>
+      <c r="B50" s="4">
+        <v>49</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J50" s="4"/>
+    </row>
+    <row r="51" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A51" s="4">
+        <v>50</v>
+      </c>
+      <c r="B51" s="4">
+        <v>50</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="I51" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J51" s="4"/>
+    </row>
+    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A52" s="4">
+        <v>51</v>
+      </c>
+      <c r="B52" s="4">
+        <v>51</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J52" s="4"/>
+    </row>
+    <row r="53" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A53" s="4">
+        <v>52</v>
+      </c>
+      <c r="B53" s="4">
+        <v>52</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="H53" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="I53" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J53" s="4"/>
+    </row>
+    <row r="54" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A54" s="4">
+        <v>53</v>
+      </c>
+      <c r="B54" s="4">
+        <v>53</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="H54" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="I54" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J54" s="4"/>
+    </row>
+    <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A55" s="4">
+        <v>54</v>
+      </c>
+      <c r="B55" s="4">
+        <v>54</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="I55" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J55" s="4"/>
+    </row>
+    <row r="56" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A56" s="4">
+        <v>55</v>
+      </c>
+      <c r="B56" s="4">
+        <v>55</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="I56" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J56" s="4"/>
+    </row>
+    <row r="57" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A57" s="4">
+        <v>56</v>
+      </c>
+      <c r="B57" s="4">
+        <v>56</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="H57" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I57" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J57" s="4"/>
+    </row>
+    <row r="58" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A58" s="4">
+        <v>57</v>
+      </c>
+      <c r="B58" s="4">
+        <v>57</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="H58" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="I58" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J58" s="4"/>
+    </row>
+    <row r="59" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A59" s="4">
+        <v>58</v>
+      </c>
+      <c r="B59" s="4">
+        <v>58</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="H59" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="I59" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J59" s="4"/>
+    </row>
+    <row r="60" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A60" s="4">
+        <v>59</v>
+      </c>
+      <c r="B60" s="4">
+        <v>59</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="G60" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="H60" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="I60" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J60" s="4"/>
+    </row>
+    <row r="61" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A61" s="4">
+        <v>60</v>
+      </c>
+      <c r="B61" s="4">
+        <v>60</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G61" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="H61" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="I61" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J61" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1"/>
-    <hyperlink ref="F7" r:id="rId2"/>
-    <hyperlink ref="F8" r:id="rId3"/>
-    <hyperlink ref="F9" r:id="rId4"/>
+    <hyperlink ref="F3" r:id="rId1"/>
+    <hyperlink ref="F8" r:id="rId2"/>
+    <hyperlink ref="F9" r:id="rId3"/>
+    <hyperlink ref="F10" r:id="rId4"/>
+    <hyperlink ref="F2" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
+  <drawing r:id="rId7"/>
+  <legacyDrawing r:id="rId8"/>
+  <controls>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="1026" r:id="rId9" name="Control 2">
+          <controlPr defaultSize="0" r:id="rId10">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>52</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>523875</xdr:colOff>
+                <xdr:row>53</xdr:row>
+                <xdr:rowOff>352425</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="1026" r:id="rId9" name="Control 2"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="1025" r:id="rId11" name="Control 1">
+          <controlPr defaultSize="0" r:id="rId10">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>52</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>514350</xdr:colOff>
+                <xdr:row>53</xdr:row>
+                <xdr:rowOff>352425</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="1025" r:id="rId11" name="Control 1"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+  </controls>
 </worksheet>
 </file>
 

</xml_diff>